<commit_message>
feat: Update database design file and remove temporary backup
</commit_message>
<xml_diff>
--- a/database/database_design.xlsx
+++ b/database/database_design.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\michi\Documents\project_one_local\2024-2025-projectone-mct-MichielGekiere\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4802E102-D889-4FE3-AC87-976B0AB75C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BDCD7C53-348F-421A-8335-B5B311D92A0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{66765D26-31D2-4853-8308-282CA887A50B}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Tables" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,6 +35,74 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="21">
+  <si>
+    <t>sensor_id</t>
+  </si>
+  <si>
+    <t>sensors</t>
+  </si>
+  <si>
+    <t>power_logs</t>
+  </si>
+  <si>
+    <t>battery_tracking</t>
+  </si>
+  <si>
+    <t>actuators</t>
+  </si>
+  <si>
+    <t>sensor_name</t>
+  </si>
+  <si>
+    <t>datetime</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>actuator_id</t>
+  </si>
+  <si>
+    <t>actuator_name</t>
+  </si>
+  <si>
+    <t>log_id</t>
+  </si>
+  <si>
+    <t>log_name</t>
+  </si>
+  <si>
+    <t>track_id</t>
+  </si>
+  <si>
+    <t>input_value</t>
+  </si>
+  <si>
+    <t>output_value</t>
+  </si>
+  <si>
+    <t>value_unit</t>
+  </si>
+  <si>
+    <t>input_unit</t>
+  </si>
+  <si>
+    <t>output_unit</t>
+  </si>
+  <si>
+    <t>user_input</t>
+  </si>
+  <si>
+    <t>input_id</t>
+  </si>
+  <si>
+    <t>input_name</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
@@ -46,18 +114,74 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0070C0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -66,8 +190,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -402,9 +536,130 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46FD3357-C0B7-4EB6-9A4F-09A461B6A0C3}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="11.6328125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.1796875" style="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14" style="8" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="C7" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add initial database schema and data for power_link project
- Created MySQL database `power_link` with UTF-8 character set.
- Defined tables: `actuators`, `inhabitants`, `inputs`, `measurements`, `sensors`, `signals`, and `user_inputs`.
- Established primary and unique keys for each table.
- Included foreign key constraints to maintain referential integrity between related tables.
- Prepared SQL dump for future data restoration and migration.
</commit_message>
<xml_diff>
--- a/database/database_design.xlsx
+++ b/database/database_design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\michi\Documents\project_one_local\2024-2025-projectone-mct-MichielGekiere\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BDCD7C53-348F-421A-8335-B5B311D92A0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F09071C-1174-4F9E-A189-B3E29DAE94A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{66765D26-31D2-4853-8308-282CA887A50B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="29">
   <si>
     <t>sensor_id</t>
   </si>
@@ -44,61 +44,85 @@
     <t>sensors</t>
   </si>
   <si>
-    <t>power_logs</t>
+    <t>actuators</t>
+  </si>
+  <si>
+    <t>sensor_name</t>
+  </si>
+  <si>
+    <t>datetime</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>actuator_id</t>
+  </si>
+  <si>
+    <t>actuator_name</t>
+  </si>
+  <si>
+    <t>value_unit</t>
+  </si>
+  <si>
+    <t>user_input</t>
+  </si>
+  <si>
+    <t>input_id</t>
+  </si>
+  <si>
+    <t>measurements</t>
+  </si>
+  <si>
+    <t>measurement_id</t>
+  </si>
+  <si>
+    <t>inputs</t>
+  </si>
+  <si>
+    <t>signals</t>
+  </si>
+  <si>
+    <t>signal_id</t>
+  </si>
+  <si>
+    <t>user_input_id</t>
+  </si>
+  <si>
+    <t>user_input_name</t>
+  </si>
+  <si>
+    <t>first_name</t>
+  </si>
+  <si>
+    <t>last_name</t>
+  </si>
+  <si>
+    <t>badge_id</t>
+  </si>
+  <si>
+    <t>inhabitant</t>
+  </si>
+  <si>
+    <t>inhabitant_id</t>
   </si>
   <si>
     <t>battery_tracking</t>
   </si>
   <si>
-    <t>actuators</t>
-  </si>
-  <si>
-    <t>sensor_name</t>
-  </si>
-  <si>
-    <t>datetime</t>
-  </si>
-  <si>
-    <t>value</t>
-  </si>
-  <si>
-    <t>actuator_id</t>
-  </si>
-  <si>
-    <t>actuator_name</t>
-  </si>
-  <si>
-    <t>log_id</t>
-  </si>
-  <si>
-    <t>log_name</t>
-  </si>
-  <si>
-    <t>track_id</t>
+    <t>tracking_id</t>
   </si>
   <si>
     <t>input_value</t>
   </si>
   <si>
+    <t>input_unit</t>
+  </si>
+  <si>
     <t>output_value</t>
   </si>
   <si>
-    <t>value_unit</t>
-  </si>
-  <si>
-    <t>input_unit</t>
-  </si>
-  <si>
     <t>output_unit</t>
-  </si>
-  <si>
-    <t>user_input</t>
-  </si>
-  <si>
-    <t>input_id</t>
-  </si>
-  <si>
-    <t>input_name</t>
   </si>
 </sst>
 </file>
@@ -114,7 +138,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -148,6 +172,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -190,9 +226,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
@@ -202,6 +237,13 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -536,127 +578,148 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46FD3357-C0B7-4EB6-9A4F-09A461B6A0C3}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.6328125" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.1796875" style="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14" style="8" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.6328125" style="14" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7265625" style="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.7265625" style="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.54296875" style="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.1796875" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10" style="7" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14" style="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="13" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" s="16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="15" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="D3" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>3</v>
+      <c r="F3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="I3" s="15" t="s">
+        <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="I4" s="15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="I5" s="15" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B6" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>12</v>
+      <c r="E6" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="I6" s="15" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C7" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>17</v>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="I7" s="15" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add initial database model for Power Link ERD
- Created a new MySQL Workbench model archive for the Power Link project.
- Included the database schema definitions for 'mydb' and 'power_link'.
- This commit establishes the foundational structure for the database design.
</commit_message>
<xml_diff>
--- a/database/database_design.xlsx
+++ b/database/database_design.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\michi\Documents\project_one_local\2024-2025-projectone-mct-MichielGekiere\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F09071C-1174-4F9E-A189-B3E29DAE94A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F13BB7E-E11D-4C22-A585-73C118DBBA5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{66765D26-31D2-4853-8308-282CA887A50B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{66765D26-31D2-4853-8308-282CA887A50B}"/>
   </bookViews>
   <sheets>
-    <sheet name="Tables" sheetId="1" r:id="rId1"/>
+    <sheet name="Version1" sheetId="3" r:id="rId1"/>
+    <sheet name="Version2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="53">
   <si>
     <t>sensor_id</t>
   </si>
@@ -101,9 +102,6 @@
     <t>badge_id</t>
   </si>
   <si>
-    <t>inhabitant</t>
-  </si>
-  <si>
     <t>inhabitant_id</t>
   </si>
   <si>
@@ -123,6 +121,81 @@
   </si>
   <si>
     <t>output_unit</t>
+  </si>
+  <si>
+    <t>inhabitants</t>
+  </si>
+  <si>
+    <t>user_input_value</t>
+  </si>
+  <si>
+    <t>heating_schedule</t>
+  </si>
+  <si>
+    <t>lighting_schedule</t>
+  </si>
+  <si>
+    <t>schedule_id</t>
+  </si>
+  <si>
+    <t>start_time</t>
+  </si>
+  <si>
+    <t>end_time</t>
+  </si>
+  <si>
+    <t>temperature</t>
+  </si>
+  <si>
+    <t>days</t>
+  </si>
+  <si>
+    <t>enabled</t>
+  </si>
+  <si>
+    <t>heater_id</t>
+  </si>
+  <si>
+    <t>ac_id</t>
+  </si>
+  <si>
+    <t>created_at</t>
+  </si>
+  <si>
+    <t>updated_at</t>
+  </si>
+  <si>
+    <t>brightness</t>
+  </si>
+  <si>
+    <t>components</t>
+  </si>
+  <si>
+    <t>schedule_types</t>
+  </si>
+  <si>
+    <t>schedules</t>
+  </si>
+  <si>
+    <t>schedule_name</t>
+  </si>
+  <si>
+    <t>type_id</t>
+  </si>
+  <si>
+    <t>type_name</t>
+  </si>
+  <si>
+    <t>component_id</t>
+  </si>
+  <si>
+    <t>component_name</t>
+  </si>
+  <si>
+    <t>component_logs</t>
+  </si>
+  <si>
+    <t>log_id</t>
   </si>
 </sst>
 </file>
@@ -188,7 +261,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -222,28 +295,86 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -577,150 +708,419 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46FD3357-C0B7-4EB6-9A4F-09A461B6A0C3}">
-  <dimension ref="A1:I7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4ED72F7-B521-4212-8200-BCF637E63C75}">
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.6328125" style="14" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.453125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7265625" style="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.7265625" style="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.54296875" style="9" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.1796875" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14" style="15" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="9" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D1" s="11" t="s">
+      <c r="C1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="I1" s="16" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="14" t="s">
+      <c r="H1" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="J1" s="13" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A2" s="10" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D2" s="12" t="s">
+      <c r="C2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="15" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" s="14" t="s">
+      <c r="H2" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="J2" s="14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="15" t="s">
+      <c r="H3" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J3" s="14" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4" s="10" t="s">
+        <v>8</v>
+      </c>
       <c r="B4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="D4" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="F4" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="I4" s="15" t="s">
+      <c r="H4" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5" s="10"/>
+      <c r="B5" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="J5" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B5" s="3" t="s">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6" s="10"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="J6" s="14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7" s="10"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="J7" s="14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" s="10"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="J8" s="14"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" s="10"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="J9" s="14"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" s="10"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="J10" s="14"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" s="10"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="I11" s="5"/>
+      <c r="J11" s="14"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAC07BD1-4258-4024-9C4C-1C3A670DDF54}">
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.453125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="B4" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" s="15"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="15"/>
+      <c r="B5" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="I5" s="15" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="B6" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="G6" s="7" t="s">
+      <c r="D5" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="E5" s="15"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="15"/>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" s="15"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="15"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7" s="15"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="15"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="15"/>
+    </row>
+    <row r="9" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="16"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="I6" s="15" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="I7" s="15" t="s">
-        <v>28</v>
-      </c>
+      <c r="E9" s="16"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" s="17"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="17"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>